<commit_message>
Update PulseGen reference spreadsheet
</commit_message>
<xml_diff>
--- a/docs/PulseGen.xlsx
+++ b/docs/PulseGen.xlsx
@@ -1,29 +1,44 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asans\Documents\Proyecto_H\Micros\Utiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andres\Labs\Projects\SmartMotion\stm32-pulse-generator\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7FA930C-F531-4544-B8CA-8758A799ABDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2C8F9F4-E26E-42F3-B34C-7B6D9A6C9D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Pulse Generator" sheetId="5" r:id="rId1"/>
+    <sheet name="Clock Config" sheetId="6" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="A10000000">#REF!</definedName>
     <definedName name="A100000000">#REF!</definedName>
     <definedName name="A4294967295">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -64,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="29">
   <si>
     <t>Timer Main Clock Frequency (CK_PSC)</t>
   </si>
@@ -136,6 +151,21 @@
   </si>
   <si>
     <t>Pulse Frequency Reslolution</t>
+  </si>
+  <si>
+    <t>Timer Counter Frequency (CK_CNT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum Pulse Frequency </t>
+  </si>
+  <si>
+    <t>Minimum Pulse Frequency</t>
+  </si>
+  <si>
+    <t>Best Frequency Resolution</t>
+  </si>
+  <si>
+    <t>Worst Frequency Resolution</t>
   </si>
 </sst>
 </file>
@@ -263,7 +293,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyProtection="1">
       <protection locked="0"/>
@@ -332,6 +362,7 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -656,33 +687,33 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C4EADBC-A422-416C-B596-3C9E42FC6D5E}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.5546875" style="12" customWidth="1"/>
+    <col min="1" max="1" width="40.5703125" style="12" customWidth="1"/>
     <col min="2" max="2" width="12" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.5546875" style="13"/>
+    <col min="3" max="3" width="11.5703125" style="13"/>
     <col min="5" max="5" width="23" customWidth="1"/>
-    <col min="6" max="6" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" style="6"/>
+    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5703125" style="6"/>
     <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="G1"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="29" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="E2" s="28" t="s">
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="E2" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="15" t="s">
         <v>0</v>
       </c>
@@ -702,12 +733,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="1">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>5</v>
@@ -723,7 +754,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="15" t="s">
         <v>12</v>
       </c>
@@ -744,7 +775,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="15" t="s">
         <v>14</v>
       </c>
@@ -765,27 +796,27 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="19"/>
       <c r="B7"/>
       <c r="C7" s="20"/>
       <c r="G7"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="19"/>
       <c r="B8"/>
       <c r="C8" s="20"/>
       <c r="G8"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="27" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
       <c r="G9"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
         <v>6</v>
       </c>
@@ -797,7 +828,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
         <v>7</v>
       </c>
@@ -809,7 +840,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
         <v>1</v>
       </c>
@@ -821,19 +852,19 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="23" t="s">
         <v>10</v>
       </c>
       <c r="B13" s="5">
         <f>2^B4-1</f>
-        <v>4294967295</v>
+        <v>65535</v>
       </c>
       <c r="C13" s="24" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
         <v>15</v>
       </c>
@@ -845,7 +876,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
         <v>16</v>
       </c>
@@ -855,19 +886,19 @@
       </c>
       <c r="C15" s="22"/>
     </row>
-    <row r="16" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="25" t="s">
         <v>17</v>
       </c>
       <c r="B16" s="5">
         <f>$B$12/$B$13/2</f>
-        <v>4.8894435178696745E-3</v>
+        <v>320.43945983062486</v>
       </c>
       <c r="C16" s="24" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
         <v>20</v>
       </c>
@@ -879,7 +910,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="26" t="s">
         <v>18</v>
       </c>
@@ -891,20 +922,19 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="26" t="s">
         <v>19</v>
       </c>
       <c r="B19" s="3">
         <f>$B$14*(1/$B$13-1/($B$13+1))</f>
-        <v>1.1384122811097797E-12</v>
+        <v>4.8895181248569293E-3</v>
       </c>
       <c r="C19" s="22" t="s">
         <v>2</v>
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="3">
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="E2:G2"/>
@@ -941,4 +971,136 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C9A04C3-89BB-4420-991A-9D16663FD1C9}">
+  <dimension ref="A3:C11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="36.140625" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1">
+        <v>16</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="27" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="27">
+        <f>2^B3-1</f>
+        <v>65535</v>
+      </c>
+      <c r="C4" s="27" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="4">
+        <v>84000000</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="4">
+        <v>83</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="27">
+        <f>B5/(B6+1)</f>
+        <v>1000000</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="27">
+        <f>B7/2</f>
+        <v>500000</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="27">
+        <f>B7/(2*(B4+1))</f>
+        <v>7.62939453125</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="27">
+        <f>B7/2*(1/(B4)-1/(B4+1))</f>
+        <v>1.1641709821087927E-4</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="27">
+        <f>B7/2*(1/1-1/2)</f>
+        <v>250000</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" operator="equal" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" xr:uid="{38753F13-8DF5-45FE-A836-E161F59A384F}">
+      <formula1>"16,32"</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="TIMx_PSC out of range" error="TIMx_PSC must be an integer between 0 and TIMxARR." sqref="B6" xr:uid="{CF9E5EA6-4657-41B0-88F3-22F711A64032}">
+      <formula1>0</formula1>
+      <formula2>B4</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="B7" unlockedFormula="1"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>